<commit_message>
Made it responsive to mobile phones, changed data a bit, added analytics
</commit_message>
<xml_diff>
--- a/Data/data.xlsx
+++ b/Data/data.xlsx
@@ -19,21 +19,21 @@
   </sheets>
   <definedNames>
     <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">Testing!$A$1:$AE$395</definedName>
-    <definedName hidden="1" localSheetId="0" name="Z_BB820615_2D56_4D51_A6B9_5A2C2956BFF0_.wvu.FilterData">General!$A$1:$AM$995</definedName>
-    <definedName hidden="1" localSheetId="1" name="Z_BB820615_2D56_4D51_A6B9_5A2C2956BFF0_.wvu.FilterData">Testing!$A$1:$AO$995</definedName>
-    <definedName hidden="1" localSheetId="0" name="Z_3115983D_7BEC_4A22_AEAF_FFE889ECBFEB_.wvu.FilterData">General!$A$1:$AB$2</definedName>
-    <definedName hidden="1" localSheetId="1" name="Z_3115983D_7BEC_4A22_AEAF_FFE889ECBFEB_.wvu.FilterData">Testing!$A$1:$AD$2</definedName>
-    <definedName hidden="1" localSheetId="0" name="Z_734104D0_0492_4257_960F_774EFA0060B3_.wvu.FilterData">General!$A$1:$AN$995</definedName>
-    <definedName hidden="1" localSheetId="1" name="Z_734104D0_0492_4257_960F_774EFA0060B3_.wvu.FilterData">Testing!$A$1:$AP$995</definedName>
-    <definedName hidden="1" localSheetId="0" name="Z_8DD1EF62_E161_41FE_A315_B3CE54A834B9_.wvu.FilterData">General!$A$1:$AC$995</definedName>
-    <definedName hidden="1" localSheetId="1" name="Z_8DD1EF62_E161_41FE_A315_B3CE54A834B9_.wvu.FilterData">Testing!$A$1:$AE$995</definedName>
+    <definedName hidden="1" localSheetId="0" name="Z_44386414_1588_42F2_9459_28B490047402_.wvu.FilterData">General!$A$1:$AB$2</definedName>
+    <definedName hidden="1" localSheetId="1" name="Z_44386414_1588_42F2_9459_28B490047402_.wvu.FilterData">Testing!$A$1:$AD$2</definedName>
+    <definedName hidden="1" localSheetId="0" name="Z_063B7EB2_069F_4F9C_A7FD_D772A13E0079_.wvu.FilterData">General!$A$1:$AN$995</definedName>
+    <definedName hidden="1" localSheetId="1" name="Z_063B7EB2_069F_4F9C_A7FD_D772A13E0079_.wvu.FilterData">Testing!$A$1:$AP$995</definedName>
+    <definedName hidden="1" localSheetId="0" name="Z_377AB903_EB63_44E3_8EC7_3926E19DB0A5_.wvu.FilterData">General!$A$1:$AC$995</definedName>
+    <definedName hidden="1" localSheetId="1" name="Z_377AB903_EB63_44E3_8EC7_3926E19DB0A5_.wvu.FilterData">Testing!$A$1:$AE$995</definedName>
+    <definedName hidden="1" localSheetId="0" name="Z_F160EC98_CA58_4056_A44B_E9138C83A4FA_.wvu.FilterData">General!$A$1:$AM$995</definedName>
+    <definedName hidden="1" localSheetId="1" name="Z_F160EC98_CA58_4056_A44B_E9138C83A4FA_.wvu.FilterData">Testing!$A$1:$AO$995</definedName>
   </definedNames>
   <calcPr/>
   <customWorkbookViews>
-    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{734104D0-0492-4257-960F-774EFA0060B3}" name="Filter 4"/>
-    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{3115983D-7BEC-4A22-AEAF-FFE889ECBFEB}" name="Filter 2"/>
-    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{BB820615-2D56-4D51-A6B9-5A2C2956BFF0}" name="Filter 3"/>
-    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{8DD1EF62-E161-41FE-A315-B3CE54A834B9}" name="Filter 1"/>
+    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{063B7EB2-069F-4F9C-A7FD-D772A13E0079}" name="Filter 4"/>
+    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{44386414-1588-42F2-9459-28B490047402}" name="Filter 2"/>
+    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{F160EC98-CA58-4056-A44B-E9138C83A4FA}" name="Filter 3"/>
+    <customWorkbookView activeSheetId="0" maximized="1" windowHeight="0" windowWidth="0" guid="{377AB903-EB63-44E3-8EC7-3926E19DB0A5}" name="Filter 1"/>
   </customWorkbookViews>
 </workbook>
 </file>
@@ -3030,7 +3030,7 @@
     </r>
   </si>
   <si>
-    <t>Did your character take a mirror selfie in insta DP</t>
+    <t>Is your character a Gym guy</t>
   </si>
   <si>
     <t>POTTANGI DILEEP KUMAR</t>
@@ -39441,13 +39441,13 @@
     </row>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{8DD1EF62-E161-41FE-A315-B3CE54A834B9}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{377AB903-EB63-44E3-8EC7-3926E19DB0A5}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$AC$995"/>
     </customSheetView>
-    <customSheetView guid="{BB820615-2D56-4D51-A6B9-5A2C2956BFF0}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{F160EC98-CA58-4056-A44B-E9138C83A4FA}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$AM$995"/>
     </customSheetView>
-    <customSheetView guid="{734104D0-0492-4257-960F-774EFA0060B3}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{063B7EB2-069F-4F9C-A7FD-D772A13E0079}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$AN$995">
         <filterColumn colId="2">
           <filters>
@@ -39482,7 +39482,7 @@
         </filterColumn>
       </autoFilter>
     </customSheetView>
-    <customSheetView guid="{3115983D-7BEC-4A22-AEAF-FFE889ECBFEB}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{44386414-1588-42F2-9459-28B490047402}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$AB$2"/>
     </customSheetView>
   </customSheetViews>
@@ -68500,16 +68500,16 @@
     </filterColumn>
   </autoFilter>
   <customSheetViews>
-    <customSheetView guid="{3115983D-7BEC-4A22-AEAF-FFE889ECBFEB}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{44386414-1588-42F2-9459-28B490047402}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$AD$2"/>
     </customSheetView>
-    <customSheetView guid="{BB820615-2D56-4D51-A6B9-5A2C2956BFF0}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{F160EC98-CA58-4056-A44B-E9138C83A4FA}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$AO$995"/>
     </customSheetView>
-    <customSheetView guid="{8DD1EF62-E161-41FE-A315-B3CE54A834B9}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{377AB903-EB63-44E3-8EC7-3926E19DB0A5}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$AE$995"/>
     </customSheetView>
-    <customSheetView guid="{734104D0-0492-4257-960F-774EFA0060B3}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{063B7EB2-069F-4F9C-A7FD-D772A13E0079}" filter="1" showAutoFilter="1">
       <autoFilter ref="$A$1:$AP$995">
         <filterColumn colId="2">
           <filters>

</xml_diff>